<commit_message>
updated the learning Note
</commit_message>
<xml_diff>
--- a/EXCEL & POWER BI LREANING/01.introduction-to-excel.xlsx
+++ b/EXCEL & POWER BI LREANING/01.introduction-to-excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28330"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Chandoo.org\Courses\FREE DA Course\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fa0cbb6b8c034a61/Documents/MY-LEARNINGS/EXCEL &amp; POWER BI LREANING/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71B8D98-5F79-49DA-B7EB-1A68616C4F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{B71B8D98-5F79-49DA-B7EB-1A68616C4F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{928CAB8A-A260-4CE5-B944-F864375E47DF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{680501D2-1D58-4043-8C51-363F2BA2A10E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{680501D2-1D58-4043-8C51-363F2BA2A10E}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -34,6 +34,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -466,9 +469,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="14"/>
       <color theme="1"/>
@@ -520,7 +523,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -862,20 +865,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF3E5D69-0126-4153-9E40-BBA6CB3C5CF3}">
   <dimension ref="A1:I58"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="8.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.09765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="3.8984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.09765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.09765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="3.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -904,7 +907,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -933,7 +936,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -962,7 +965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -991,7 +994,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1020,7 +1023,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -1049,7 +1052,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1078,7 +1081,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -1107,7 +1110,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1136,7 +1139,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -1165,7 +1168,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -1194,7 +1197,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -1223,7 +1226,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -1252,7 +1255,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -1281,7 +1284,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>48</v>
       </c>
@@ -1310,7 +1313,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -1339,7 +1342,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>54</v>
       </c>
@@ -1368,7 +1371,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>57</v>
       </c>
@@ -1397,7 +1400,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>60</v>
       </c>
@@ -1426,7 +1429,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>63</v>
       </c>
@@ -1455,7 +1458,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>65</v>
       </c>
@@ -1484,7 +1487,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>68</v>
       </c>
@@ -1513,7 +1516,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>70</v>
       </c>
@@ -1542,7 +1545,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>72</v>
       </c>
@@ -1571,7 +1574,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>74</v>
       </c>
@@ -1600,7 +1603,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -1629,7 +1632,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>76</v>
       </c>
@@ -1658,7 +1661,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>78</v>
       </c>
@@ -1687,7 +1690,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -1716,7 +1719,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>83</v>
       </c>
@@ -1745,7 +1748,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>85</v>
       </c>
@@ -1774,7 +1777,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
         <v>87</v>
       </c>
@@ -1803,7 +1806,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
         <v>90</v>
       </c>
@@ -1832,7 +1835,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
         <v>92</v>
       </c>
@@ -1861,7 +1864,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9">
       <c r="A35" t="s">
         <v>94</v>
       </c>
@@ -1890,7 +1893,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
         <v>96</v>
       </c>
@@ -1919,7 +1922,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9">
       <c r="A37" t="s">
         <v>98</v>
       </c>
@@ -1948,7 +1951,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
         <v>100</v>
       </c>
@@ -1977,7 +1980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9">
       <c r="A39" t="s">
         <v>102</v>
       </c>
@@ -2006,7 +2009,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
         <v>104</v>
       </c>
@@ -2035,7 +2038,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9">
       <c r="A41" t="s">
         <v>106</v>
       </c>
@@ -2064,7 +2067,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9">
       <c r="A42" t="s">
         <v>108</v>
       </c>
@@ -2093,7 +2096,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9">
       <c r="A43" t="s">
         <v>110</v>
       </c>
@@ -2122,7 +2125,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9">
       <c r="A44" t="s">
         <v>112</v>
       </c>
@@ -2151,7 +2154,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9">
       <c r="A45" t="s">
         <v>114</v>
       </c>
@@ -2180,7 +2183,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9">
       <c r="A46" t="s">
         <v>114</v>
       </c>
@@ -2209,7 +2212,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9">
       <c r="A47" t="s">
         <v>117</v>
       </c>
@@ -2238,7 +2241,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9">
       <c r="A48" t="s">
         <v>119</v>
       </c>
@@ -2267,7 +2270,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9">
       <c r="A49" t="s">
         <v>121</v>
       </c>
@@ -2296,7 +2299,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9">
       <c r="A50" t="s">
         <v>123</v>
       </c>
@@ -2325,7 +2328,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9">
       <c r="A51" t="s">
         <v>125</v>
       </c>
@@ -2354,7 +2357,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9">
       <c r="A52" t="s">
         <v>126</v>
       </c>
@@ -2383,7 +2386,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9">
       <c r="A53" t="s">
         <v>128</v>
       </c>
@@ -2412,7 +2415,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9">
       <c r="A54" t="s">
         <v>130</v>
       </c>
@@ -2438,7 +2441,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9">
       <c r="A55" t="s">
         <v>132</v>
       </c>
@@ -2467,7 +2470,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9">
       <c r="A56" t="s">
         <v>134</v>
       </c>
@@ -2496,7 +2499,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9">
       <c r="A57" t="s">
         <v>136</v>
       </c>
@@ -2525,7 +2528,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9">
       <c r="A58" t="s">
         <v>138</v>
       </c>

</xml_diff>